<commit_message>
Test plan: add-to-event coverage, managed-child gap, Super Admin menu/roles fixes
- PT25: participant added to an event is notified + it shows in schedule.
- PE24/PE25: managed child can't be added by email (guardian signs up).
- SA19: Super Admin add-a-participant-by-email from the roster.
- SA1 menu now lists Award Thresholds + Audit Log; SA3 lists all roles;
  SA17 reflects per-role password auto-fill and no browser autofill.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q73NfVvLQA4dcJhV7BBvZL
</commit_message>
<xml_diff>
--- a/MedinaCares_Test_Plan.xlsx
+++ b/MedinaCares_Test_Plan.xlsx
@@ -2205,7 +2205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="54" min="1" max="1"/>
@@ -3098,6 +3098,1122 @@
       <c r="G35" s="64" t="n"/>
       <c r="H35" s="64" t="n"/>
     </row>
+    <row r="36" ht="42" customHeight="1" s="54">
+      <c r="A36" s="62" t="inlineStr">
+        <is>
+          <t>PT25</t>
+        </is>
+      </c>
+      <c r="B36" s="63" t="inlineStr">
+        <is>
+          <t>As a participant, when a supervisor/admin adds me to an event, I'm notified and it shows in my schedule.</t>
+        </is>
+      </c>
+      <c r="C36" s="63" t="inlineStr">
+        <is>
+          <t>Have a supervisor or Super Admin add your account email to an event → then open your dashboard/My sign-ups.</t>
+        </is>
+      </c>
+      <c r="D36" s="63" t="inlineStr">
+        <is>
+          <t>You (and your parent, if a parent email is on file) receive an 'added to &lt;event&gt;' email; the event appears in your upcoming sign-ups.</t>
+        </is>
+      </c>
+      <c r="E36" s="64" t="n"/>
+      <c r="F36" s="64" t="n"/>
+      <c r="G36" s="64" t="n"/>
+      <c r="H36" s="64" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" s="54">
+      <c r="A37" s="61" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="B37" s="59" t="n"/>
+      <c r="C37" s="59" t="n"/>
+      <c r="D37" s="59" t="n"/>
+      <c r="E37" s="59" t="n"/>
+      <c r="F37" s="59" t="n"/>
+      <c r="G37" s="59" t="n"/>
+      <c r="H37" s="59" t="n"/>
+    </row>
+    <row r="38" ht="42" customHeight="1" s="54">
+      <c r="A38" s="62" t="inlineStr">
+        <is>
+          <t>X1</t>
+        </is>
+      </c>
+      <c r="B38" s="63" t="inlineStr">
+        <is>
+          <t>As a phone user, I want a usable mobile layout.</t>
+        </is>
+      </c>
+      <c r="C38" s="63" t="inlineStr">
+        <is>
+          <t>Open at phone width; use the menu drawer.</t>
+        </is>
+      </c>
+      <c r="D38" s="63" t="inlineStr">
+        <is>
+          <t>Layout adapts; drawer opens/closes; no horizontal scroll.</t>
+        </is>
+      </c>
+      <c r="E38" s="64" t="n"/>
+      <c r="F38" s="64" t="n"/>
+      <c r="G38" s="64" t="n"/>
+      <c r="H38" s="64" t="n"/>
+    </row>
+    <row r="39" ht="42" customHeight="1" s="54">
+      <c r="A39" s="62" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="B39" s="63" t="inlineStr">
+        <is>
+          <t>As a visitor, I want the recycling ribbon on the login page.</t>
+        </is>
+      </c>
+      <c r="C39" s="63" t="inlineStr">
+        <is>
+          <t>Open login signed out.</t>
+        </is>
+      </c>
+      <c r="D39" s="63" t="inlineStr">
+        <is>
+          <t>Green ribbon shows on login.</t>
+        </is>
+      </c>
+      <c r="E39" s="64" t="n"/>
+      <c r="F39" s="64" t="n"/>
+      <c r="G39" s="64" t="n"/>
+      <c r="H39" s="64" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E4:E39">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
+      <formula>"Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G39">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E4:E39 G4:G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Blocked,Not tested,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="54" min="1" max="1"/>
+    <col width="56" customWidth="1" style="54" min="2" max="2"/>
+    <col width="50" customWidth="1" style="54" min="3" max="3"/>
+    <col width="50" customWidth="1" style="54" min="4" max="4"/>
+    <col width="13" customWidth="1" style="54" min="5" max="5"/>
+    <col width="30" customWidth="1" style="54" min="6" max="6"/>
+    <col width="13" customWidth="1" style="54" min="7" max="7"/>
+    <col width="30" customWidth="1" style="54" min="8" max="8"/>
+    <col width="13" customWidth="1" style="54" min="9" max="9"/>
+    <col width="30" customWidth="1" style="54" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" s="54">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>Test cases — Parent — elementary (2–5 child)</t>
+        </is>
+      </c>
+      <c r="B1" s="57" t="n"/>
+      <c r="C1" s="57" t="n"/>
+      <c r="D1" s="57" t="n"/>
+      <c r="E1" s="57" t="n"/>
+      <c r="F1" s="57" t="n"/>
+      <c r="G1" s="57" t="n"/>
+      <c r="H1" s="57" t="n"/>
+      <c r="I1" s="57" t="n"/>
+      <c r="J1" s="57" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="54">
+      <c r="E2" s="58" t="inlineStr">
+        <is>
+          <t>Noreen Sultana
+Platform: ?</t>
+        </is>
+      </c>
+      <c r="F2" s="59" t="n"/>
+      <c r="G2" s="58" t="inlineStr">
+        <is>
+          <t>Tester 2
+Platform: ?</t>
+        </is>
+      </c>
+      <c r="H2" s="59" t="n"/>
+      <c r="I2" s="58" t="inlineStr">
+        <is>
+          <t>Tester 3
+Platform: ?</t>
+        </is>
+      </c>
+      <c r="J2" s="59" t="n"/>
+    </row>
+    <row r="3" ht="28" customHeight="1" s="54">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="60" t="inlineStr">
+        <is>
+          <t>User story</t>
+        </is>
+      </c>
+      <c r="C3" s="60" t="inlineStr">
+        <is>
+          <t>Steps to perform</t>
+        </is>
+      </c>
+      <c r="D3" s="60" t="inlineStr">
+        <is>
+          <t>Expected behavior (what you should see)</t>
+        </is>
+      </c>
+      <c r="E3" s="60" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="F3" s="60" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="G3" s="60" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="H3" s="60" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="I3" s="60" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="J3" s="60" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" s="54">
+      <c r="A4" s="61" t="inlineStr">
+        <is>
+          <t>Account &amp; access (all roles)</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="n"/>
+      <c r="C4" s="59" t="n"/>
+      <c r="D4" s="59" t="n"/>
+      <c r="E4" s="59" t="n"/>
+      <c r="F4" s="59" t="n"/>
+      <c r="G4" s="59" t="n"/>
+      <c r="H4" s="59" t="n"/>
+      <c r="I4" s="59" t="n"/>
+      <c r="J4" s="59" t="n"/>
+    </row>
+    <row r="5" ht="42" customHeight="1" s="54">
+      <c r="A5" s="62" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>As any user, I want to log in with email and password.</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>Enter valid email/password and Sign in.</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>You're signed in and taken to your role's home.</t>
+        </is>
+      </c>
+      <c r="E5" s="64" t="n"/>
+      <c r="F5" s="64" t="n"/>
+      <c r="G5" s="64" t="n"/>
+      <c r="H5" s="64" t="n"/>
+      <c r="I5" s="64" t="n"/>
+      <c r="J5" s="64" t="n"/>
+    </row>
+    <row r="6" ht="42" customHeight="1" s="54">
+      <c r="A6" s="62" t="inlineStr">
+        <is>
+          <t>AC2</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>As any user, I want to reveal my password while typing.</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>Tap the eye icon in the password field.</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>Password text toggles visible/hidden.</t>
+        </is>
+      </c>
+      <c r="E6" s="64" t="n"/>
+      <c r="F6" s="64" t="n"/>
+      <c r="G6" s="64" t="n"/>
+      <c r="H6" s="64" t="n"/>
+      <c r="I6" s="64" t="n"/>
+      <c r="J6" s="64" t="n"/>
+    </row>
+    <row r="7" ht="42" customHeight="1" s="54">
+      <c r="A7" s="62" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B7" s="63" t="inlineStr">
+        <is>
+          <t>As any user, I want to reset a forgotten password by email.</t>
+        </is>
+      </c>
+      <c r="C7" s="63" t="inlineStr">
+        <is>
+          <t>Forgot password → enter email → open email → follow link → set new password → sign in.</t>
+        </is>
+      </c>
+      <c r="D7" s="63" t="inlineStr">
+        <is>
+          <t>Reset email arrives; link works; new password signs in; old one fails.</t>
+        </is>
+      </c>
+      <c r="E7" s="64" t="n"/>
+      <c r="F7" s="64" t="n"/>
+      <c r="G7" s="64" t="n"/>
+      <c r="H7" s="64" t="n"/>
+      <c r="I7" s="64" t="n"/>
+      <c r="J7" s="64" t="n"/>
+    </row>
+    <row r="8" ht="42" customHeight="1" s="54">
+      <c r="A8" s="62" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="B8" s="63" t="inlineStr">
+        <is>
+          <t>As any user, I want to sign out.</t>
+        </is>
+      </c>
+      <c r="C8" s="63" t="inlineStr">
+        <is>
+          <t>Use Sign out.</t>
+        </is>
+      </c>
+      <c r="D8" s="63" t="inlineStr">
+        <is>
+          <t>Logged out; returned to login/landing.</t>
+        </is>
+      </c>
+      <c r="E8" s="64" t="n"/>
+      <c r="F8" s="64" t="n"/>
+      <c r="G8" s="64" t="n"/>
+      <c r="H8" s="64" t="n"/>
+      <c r="I8" s="64" t="n"/>
+      <c r="J8" s="64" t="n"/>
+    </row>
+    <row r="9" ht="42" customHeight="1" s="54">
+      <c r="A9" s="62" t="inlineStr">
+        <is>
+          <t>AC5</t>
+        </is>
+      </c>
+      <c r="B9" s="63" t="inlineStr">
+        <is>
+          <t>As any user, I want a clear error for bad credentials.</t>
+        </is>
+      </c>
+      <c r="C9" s="63" t="inlineStr">
+        <is>
+          <t>Enter a wrong password.</t>
+        </is>
+      </c>
+      <c r="D9" s="63" t="inlineStr">
+        <is>
+          <t>Clear 'login failed' message; stay on login.</t>
+        </is>
+      </c>
+      <c r="E9" s="64" t="n"/>
+      <c r="F9" s="64" t="n"/>
+      <c r="G9" s="64" t="n"/>
+      <c r="H9" s="64" t="n"/>
+      <c r="I9" s="64" t="n"/>
+      <c r="J9" s="64" t="n"/>
+    </row>
+    <row r="10" ht="42" customHeight="1" s="54">
+      <c r="A10" s="62" t="inlineStr">
+        <is>
+          <t>AC6</t>
+        </is>
+      </c>
+      <c r="B10" s="63" t="inlineStr">
+        <is>
+          <t>As any user, my session persists and protected pages are guarded.</t>
+        </is>
+      </c>
+      <c r="C10" s="63" t="inlineStr">
+        <is>
+          <t>Sign in, refresh; then sign out and open a protected URL directly.</t>
+        </is>
+      </c>
+      <c r="D10" s="63" t="inlineStr">
+        <is>
+          <t>Refresh stays signed in; protected pages redirect to login when signed out.</t>
+        </is>
+      </c>
+      <c r="E10" s="64" t="n"/>
+      <c r="F10" s="64" t="n"/>
+      <c r="G10" s="64" t="n"/>
+      <c r="H10" s="64" t="n"/>
+      <c r="I10" s="64" t="n"/>
+      <c r="J10" s="64" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" s="54">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>Parent — elementary (grades 2–5 child)</t>
+        </is>
+      </c>
+      <c r="B11" s="59" t="n"/>
+      <c r="C11" s="59" t="n"/>
+      <c r="D11" s="59" t="n"/>
+      <c r="E11" s="59" t="n"/>
+      <c r="F11" s="59" t="n"/>
+      <c r="G11" s="59" t="n"/>
+      <c r="H11" s="59" t="n"/>
+      <c r="I11" s="59" t="n"/>
+      <c r="J11" s="59" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1" s="54">
+      <c r="A12" s="62" t="inlineStr">
+        <is>
+          <t>PE1</t>
+        </is>
+      </c>
+      <c r="B12" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to register to manage my grade 2–5 child.</t>
+        </is>
+      </c>
+      <c r="C12" s="63" t="inlineStr">
+        <is>
+          <t>Create account → parent of a 2–5 child.</t>
+        </is>
+      </c>
+      <c r="D12" s="63" t="inlineStr">
+        <is>
+          <t>Parent account created.</t>
+        </is>
+      </c>
+      <c r="E12" s="64" t="n"/>
+      <c r="F12" s="64" t="n"/>
+      <c r="G12" s="64" t="n"/>
+      <c r="H12" s="64" t="n"/>
+      <c r="I12" s="64" t="n"/>
+      <c r="J12" s="64" t="n"/>
+    </row>
+    <row r="13" ht="42" customHeight="1" s="54">
+      <c r="A13" s="62" t="inlineStr">
+        <is>
+          <t>PE2</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>As an elementary parent, I want the right menu tabs.</t>
+        </is>
+      </c>
+      <c r="C13" s="63" t="inlineStr">
+        <is>
+          <t>Look at the left menu.</t>
+        </is>
+      </c>
+      <c r="D13" s="63" t="inlineStr">
+        <is>
+          <t>Dashboard and Find Opportunities (Help in footer).</t>
+        </is>
+      </c>
+      <c r="E13" s="64" t="n"/>
+      <c r="F13" s="64" t="n"/>
+      <c r="G13" s="64" t="n"/>
+      <c r="H13" s="64" t="n"/>
+      <c r="I13" s="64" t="n"/>
+      <c r="J13" s="64" t="n"/>
+    </row>
+    <row r="14" ht="42" customHeight="1" s="54">
+      <c r="A14" s="62" t="inlineStr">
+        <is>
+          <t>PE3</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to add a managed child (2–5).</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>Add child with name and grade (join code if required).</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>Child added; no separate login.</t>
+        </is>
+      </c>
+      <c r="E14" s="64" t="n"/>
+      <c r="F14" s="64" t="n"/>
+      <c r="G14" s="64" t="n"/>
+      <c r="H14" s="64" t="n"/>
+      <c r="I14" s="64" t="n"/>
+      <c r="J14" s="64" t="n"/>
+    </row>
+    <row r="15" ht="42" customHeight="1" s="54">
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>PE4</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>As a parent with several kids, I want to switch child.</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>Use the child picker.</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>Selected child's context is used.</t>
+        </is>
+      </c>
+      <c r="E15" s="64" t="n"/>
+      <c r="F15" s="64" t="n"/>
+      <c r="G15" s="64" t="n"/>
+      <c r="H15" s="64" t="n"/>
+      <c r="I15" s="64" t="n"/>
+      <c r="J15" s="64" t="n"/>
+    </row>
+    <row r="16" ht="42" customHeight="1" s="54">
+      <c r="A16" s="62" t="inlineStr">
+        <is>
+          <t>PE5</t>
+        </is>
+      </c>
+      <c r="B16" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to sign my child up.</t>
+        </is>
+      </c>
+      <c r="C16" s="63" t="inlineStr">
+        <is>
+          <t>Find Opportunities → pick child → open event → sign up.</t>
+        </is>
+      </c>
+      <c r="D16" s="63" t="inlineStr">
+        <is>
+          <t>Child registered; appears on dashboard with calendar.</t>
+        </is>
+      </c>
+      <c r="E16" s="64" t="n"/>
+      <c r="F16" s="64" t="n"/>
+      <c r="G16" s="64" t="n"/>
+      <c r="H16" s="64" t="n"/>
+      <c r="I16" s="64" t="n"/>
+      <c r="J16" s="64" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1" s="54">
+      <c r="A17" s="62" t="inlineStr">
+        <is>
+          <t>PE6</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, child sign-up respects grade/org limits.</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="inlineStr">
+        <is>
+          <t>Try an ineligible event.</t>
+        </is>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>Hidden or blocked with a message.</t>
+        </is>
+      </c>
+      <c r="E17" s="64" t="n"/>
+      <c r="F17" s="64" t="n"/>
+      <c r="G17" s="64" t="n"/>
+      <c r="H17" s="64" t="n"/>
+      <c r="I17" s="64" t="n"/>
+      <c r="J17" s="64" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1" s="54">
+      <c r="A18" s="62" t="inlineStr">
+        <is>
+          <t>PE7</t>
+        </is>
+      </c>
+      <c r="B18" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to see my child's schedule.</t>
+        </is>
+      </c>
+      <c r="C18" s="63" t="inlineStr">
+        <is>
+          <t>Open the dashboard.</t>
+        </is>
+      </c>
+      <c r="D18" s="63" t="inlineStr">
+        <is>
+          <t>Child's upcoming events with add-to-calendar; new sign-ups flagged.</t>
+        </is>
+      </c>
+      <c r="E18" s="64" t="n"/>
+      <c r="F18" s="64" t="n"/>
+      <c r="G18" s="64" t="n"/>
+      <c r="H18" s="64" t="n"/>
+      <c r="I18" s="64" t="n"/>
+      <c r="J18" s="64" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1" s="54">
+      <c r="A19" s="62" t="inlineStr">
+        <is>
+          <t>PE8</t>
+        </is>
+      </c>
+      <c r="B19" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to invite a co-guardian.</t>
+        </is>
+      </c>
+      <c r="C19" s="63" t="inlineStr">
+        <is>
+          <t>Invite a co-guardian by email.</t>
+        </is>
+      </c>
+      <c r="D19" s="63" t="inlineStr">
+        <is>
+          <t>Invite email sent; on registering with that email they share access.</t>
+        </is>
+      </c>
+      <c r="E19" s="64" t="n"/>
+      <c r="F19" s="64" t="n"/>
+      <c r="G19" s="64" t="n"/>
+      <c r="H19" s="64" t="n"/>
+      <c r="I19" s="64" t="n"/>
+      <c r="J19" s="64" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1" s="54">
+      <c r="A20" s="62" t="inlineStr">
+        <is>
+          <t>PE9</t>
+        </is>
+      </c>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want notice when my child signs up.</t>
+        </is>
+      </c>
+      <c r="C20" s="63" t="inlineStr">
+        <is>
+          <t>Sign a child up (or have the other guardian do it).</t>
+        </is>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>A notification/confirmation is produced.</t>
+        </is>
+      </c>
+      <c r="E20" s="64" t="n"/>
+      <c r="F20" s="64" t="n"/>
+      <c r="G20" s="64" t="n"/>
+      <c r="H20" s="64" t="n"/>
+      <c r="I20" s="64" t="n"/>
+      <c r="J20" s="64" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1" s="54">
+      <c r="A21" s="62" t="inlineStr">
+        <is>
+          <t>PE10</t>
+        </is>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to submit my child's hours after an event (child has no login).</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>Dashboard → the child's 'Submit hours (past events)' → enter hours → Submit.</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr">
+        <is>
+          <t>Hours go to the supervisor for approval; status shows 'Waiting for review'.</t>
+        </is>
+      </c>
+      <c r="E21" s="64" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="64" t="n"/>
+      <c r="H21" s="64" t="n"/>
+      <c r="I21" s="64" t="n"/>
+      <c r="J21" s="64" t="n"/>
+    </row>
+    <row r="22" ht="42" customHeight="1" s="54">
+      <c r="A22" s="62" t="inlineStr">
+        <is>
+          <t>PE11</t>
+        </is>
+      </c>
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to resubmit my child's rejected hours.</t>
+        </is>
+      </c>
+      <c r="C22" s="63" t="inlineStr">
+        <is>
+          <t>On a rejected past event, enter corrected hours → Resubmit.</t>
+        </is>
+      </c>
+      <c r="D22" s="63" t="inlineStr">
+        <is>
+          <t>Returns to 'Waiting for review'.</t>
+        </is>
+      </c>
+      <c r="E22" s="64" t="n"/>
+      <c r="F22" s="64" t="n"/>
+      <c r="G22" s="64" t="n"/>
+      <c r="H22" s="64" t="n"/>
+      <c r="I22" s="64" t="n"/>
+      <c r="J22" s="64" t="n"/>
+    </row>
+    <row r="23" ht="42" customHeight="1" s="54">
+      <c r="A23" s="62" t="inlineStr">
+        <is>
+          <t>PE12</t>
+        </is>
+      </c>
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to see each past event's hours status for my child.</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>Look at the child's past events list.</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>Each shows Approved / Waiting / Rejected as appropriate.</t>
+        </is>
+      </c>
+      <c r="E23" s="64" t="n"/>
+      <c r="F23" s="64" t="n"/>
+      <c r="G23" s="64" t="n"/>
+      <c r="H23" s="64" t="n"/>
+      <c r="I23" s="64" t="n"/>
+      <c r="J23" s="64" t="n"/>
+    </row>
+    <row r="24" ht="42" customHeight="1" s="54">
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>PE13</t>
+        </is>
+      </c>
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, all core participant actions are available to me for my child.</t>
+        </is>
+      </c>
+      <c r="C24" s="63" t="inlineStr">
+        <is>
+          <t>Confirm: browse, sign up, withdraw, add-to-calendar, submit hours, view progress toward medals.</t>
+        </is>
+      </c>
+      <c r="D24" s="63" t="inlineStr">
+        <is>
+          <t>All participant-style actions work on the child's behalf (the child never logs in).</t>
+        </is>
+      </c>
+      <c r="E24" s="64" t="n"/>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="64" t="n"/>
+      <c r="H24" s="64" t="n"/>
+      <c r="I24" s="64" t="n"/>
+      <c r="J24" s="64" t="n"/>
+    </row>
+    <row r="25" ht="42" customHeight="1" s="54">
+      <c r="A25" s="62" t="inlineStr">
+        <is>
+          <t>PE16</t>
+        </is>
+      </c>
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to browse/search opportunities for my child (upcoming &amp; past).</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>Find Opportunities with the child selected; use search and the upcoming/past views.</t>
+        </is>
+      </c>
+      <c r="D25" s="63" t="inlineStr">
+        <is>
+          <t>Same event list a participant sees, scoped to the child's grade/org.</t>
+        </is>
+      </c>
+      <c r="E25" s="64" t="n"/>
+      <c r="F25" s="64" t="n"/>
+      <c r="G25" s="64" t="n"/>
+      <c r="H25" s="64" t="n"/>
+      <c r="I25" s="64" t="n"/>
+      <c r="J25" s="64" t="n"/>
+    </row>
+    <row r="26" ht="42" customHeight="1" s="54">
+      <c r="A26" s="62" t="inlineStr">
+        <is>
+          <t>PE17</t>
+        </is>
+      </c>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to withdraw my child from an event.</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>Open the child's upcoming events → withdraw.</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>The child is removed; the slot frees up.</t>
+        </is>
+      </c>
+      <c r="E26" s="64" t="n"/>
+      <c r="F26" s="64" t="n"/>
+      <c r="G26" s="64" t="n"/>
+      <c r="H26" s="64" t="n"/>
+      <c r="I26" s="64" t="n"/>
+      <c r="J26" s="64" t="n"/>
+    </row>
+    <row r="27" ht="42" customHeight="1" s="54">
+      <c r="A27" s="62" t="inlineStr">
+        <is>
+          <t>PE18</t>
+        </is>
+      </c>
+      <c r="B27" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to check my child in on event day.</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>On the event day within the window, check the child in.</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>Check-in succeeds for the child.</t>
+        </is>
+      </c>
+      <c r="E27" s="64" t="n"/>
+      <c r="F27" s="64" t="n"/>
+      <c r="G27" s="64" t="n"/>
+      <c r="H27" s="64" t="n"/>
+      <c r="I27" s="64" t="n"/>
+      <c r="J27" s="64" t="n"/>
+    </row>
+    <row r="28" ht="42" customHeight="1" s="54">
+      <c r="A28" s="62" t="inlineStr">
+        <is>
+          <t>PE19</t>
+        </is>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to see my child's medal progress.</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>Open the dashboard / child card.</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>Progress uses the child's grade-based thresholds (e.g. lower bar for younger grades).</t>
+        </is>
+      </c>
+      <c r="E28" s="64" t="n"/>
+      <c r="F28" s="64" t="n"/>
+      <c r="G28" s="64" t="n"/>
+      <c r="H28" s="64" t="n"/>
+      <c r="I28" s="64" t="n"/>
+      <c r="J28" s="64" t="n"/>
+    </row>
+    <row r="29" ht="42" customHeight="1" s="54">
+      <c r="A29" s="62" t="inlineStr">
+        <is>
+          <t>PE20</t>
+        </is>
+      </c>
+      <c r="B29" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, external &gt;5h for my child requires proof.</t>
+        </is>
+      </c>
+      <c r="C29" s="63" t="inlineStr">
+        <is>
+          <t>Outside hours for the child, over 5 hours, without then with a proof file.</t>
+        </is>
+      </c>
+      <c r="D29" s="63" t="inlineStr">
+        <is>
+          <t>Blocked without proof; submits with a photo/letter.</t>
+        </is>
+      </c>
+      <c r="E29" s="64" t="n"/>
+      <c r="F29" s="64" t="n"/>
+      <c r="G29" s="64" t="n"/>
+      <c r="H29" s="64" t="n"/>
+      <c r="I29" s="64" t="n"/>
+      <c r="J29" s="64" t="n"/>
+    </row>
+    <row r="30" ht="42" customHeight="1" s="54">
+      <c r="A30" s="62" t="inlineStr">
+        <is>
+          <t>PE14</t>
+        </is>
+      </c>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to log my child's outside/nonprofit volunteering.</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="inlineStr">
+        <is>
+          <t>Child card → 'Outside hours' → fill activity, org, date, hours, supervisor → Submit.</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>External hours submitted for the child and sent for supervisor approval (proof required over 5h).</t>
+        </is>
+      </c>
+      <c r="E30" s="64" t="n"/>
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="64" t="n"/>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="64" t="n"/>
+      <c r="J30" s="64" t="n"/>
+    </row>
+    <row r="31" ht="42" customHeight="1" s="54">
+      <c r="A31" s="62" t="inlineStr">
+        <is>
+          <t>PE15</t>
+        </is>
+      </c>
+      <c r="B31" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want my child's verified service record.</t>
+        </is>
+      </c>
+      <c r="C31" s="63" t="inlineStr">
+        <is>
+          <t>Child card → 'Service record'.</t>
+        </is>
+      </c>
+      <c r="D31" s="63" t="inlineStr">
+        <is>
+          <t>The child's itemized record opens; Print / Save-as-PDF works.</t>
+        </is>
+      </c>
+      <c r="E31" s="64" t="n"/>
+      <c r="F31" s="64" t="n"/>
+      <c r="G31" s="64" t="n"/>
+      <c r="H31" s="64" t="n"/>
+      <c r="I31" s="64" t="n"/>
+      <c r="J31" s="64" t="n"/>
+    </row>
+    <row r="32" ht="42" customHeight="1" s="54">
+      <c r="A32" s="62" t="inlineStr">
+        <is>
+          <t>PE22</t>
+        </is>
+      </c>
+      <c r="B32" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to be emailed when my child's hours are reviewed.</t>
+        </is>
+      </c>
+      <c r="C32" s="63" t="inlineStr">
+        <is>
+          <t>Have a supervisor approve then reject a submission for a managed child.</t>
+        </is>
+      </c>
+      <c r="D32" s="63" t="inlineStr">
+        <is>
+          <t>You (the guardian) receive the approved / needs-attention emails, even though the child has no email of their own.</t>
+        </is>
+      </c>
+      <c r="E32" s="64" t="n"/>
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="64" t="n"/>
+      <c r="H32" s="64" t="n"/>
+      <c r="I32" s="64" t="n"/>
+      <c r="J32" s="64" t="n"/>
+    </row>
+    <row r="33" ht="42" customHeight="1" s="54">
+      <c r="A33" s="62" t="inlineStr">
+        <is>
+          <t>PE23</t>
+        </is>
+      </c>
+      <c r="B33" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I want to edit my child's details.</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
+        <is>
+          <t>Child card → Edit → change name/grade/school → save.</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>Changes save for the managed child.</t>
+        </is>
+      </c>
+      <c r="E33" s="64" t="n"/>
+      <c r="F33" s="64" t="n"/>
+      <c r="G33" s="64" t="n"/>
+      <c r="H33" s="64" t="n"/>
+      <c r="I33" s="64" t="n"/>
+      <c r="J33" s="64" t="n"/>
+    </row>
+    <row r="34" ht="42" customHeight="1" s="54">
+      <c r="A34" s="62" t="inlineStr">
+        <is>
+          <t>PE24</t>
+        </is>
+      </c>
+      <c r="B34" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, I understand a managed child can't be added to an event by a supervisor's by-email tool.</t>
+        </is>
+      </c>
+      <c r="C34" s="63" t="inlineStr">
+        <is>
+          <t>Ask a supervisor/admin to try adding the child via Roster → Add a participant; then sign the child up yourself from Find Opportunities.</t>
+        </is>
+      </c>
+      <c r="D34" s="63" t="inlineStr">
+        <is>
+          <t>The by-email add can't find the child (no login/email of their own); the supported path is the guardian signing the child up, which puts the event on the child's schedule.</t>
+        </is>
+      </c>
+      <c r="E34" s="64" t="n"/>
+      <c r="F34" s="64" t="n"/>
+      <c r="G34" s="64" t="n"/>
+      <c r="H34" s="64" t="n"/>
+      <c r="I34" s="64" t="n"/>
+      <c r="J34" s="64" t="n"/>
+    </row>
+    <row r="35" ht="42" customHeight="1" s="54">
+      <c r="A35" s="62" t="inlineStr">
+        <is>
+          <t>PE25</t>
+        </is>
+      </c>
+      <c r="B35" s="63" t="inlineStr">
+        <is>
+          <t>As a parent, when I sign my child up, it appears on the child's schedule.</t>
+        </is>
+      </c>
+      <c r="C35" s="63" t="inlineStr">
+        <is>
+          <t>Find Opportunities → pick child → sign up → open dashboard.</t>
+        </is>
+      </c>
+      <c r="D35" s="63" t="inlineStr">
+        <is>
+          <t>The event shows on the child's upcoming schedule with add-to-calendar; a new-sign-up flag/confirmation appears.</t>
+        </is>
+      </c>
+      <c r="E35" s="64" t="n"/>
+      <c r="F35" s="64" t="n"/>
+      <c r="G35" s="64" t="n"/>
+      <c r="H35" s="64" t="n"/>
+      <c r="I35" s="64" t="n"/>
+      <c r="J35" s="64" t="n"/>
+    </row>
     <row r="36" ht="20" customHeight="1" s="54">
       <c r="A36" s="61" t="inlineStr">
         <is>
@@ -3111,6 +4227,8 @@
       <c r="F36" s="59" t="n"/>
       <c r="G36" s="59" t="n"/>
       <c r="H36" s="59" t="n"/>
+      <c r="I36" s="59" t="n"/>
+      <c r="J36" s="59" t="n"/>
     </row>
     <row r="37" ht="42" customHeight="1" s="54">
       <c r="A37" s="62" t="inlineStr">
@@ -3137,6 +4255,8 @@
       <c r="F37" s="64" t="n"/>
       <c r="G37" s="64" t="n"/>
       <c r="H37" s="64" t="n"/>
+      <c r="I37" s="64" t="n"/>
+      <c r="J37" s="64" t="n"/>
     </row>
     <row r="38" ht="42" customHeight="1" s="54">
       <c r="A38" s="62" t="inlineStr">
@@ -3163,15 +4283,18 @@
       <c r="F38" s="64" t="n"/>
       <c r="G38" s="64" t="n"/>
       <c r="H38" s="64" t="n"/>
+      <c r="I38" s="64" t="n"/>
+      <c r="J38" s="64" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A4:H4"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A36:J36"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A11:J11"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:E38">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
@@ -3195,1048 +4318,7 @@
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="E4:E38 G4:G38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pass,Fail,Blocked,Not tested,N/A"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" style="54" min="1" max="1"/>
-    <col width="56" customWidth="1" style="54" min="2" max="2"/>
-    <col width="50" customWidth="1" style="54" min="3" max="3"/>
-    <col width="50" customWidth="1" style="54" min="4" max="4"/>
-    <col width="13" customWidth="1" style="54" min="5" max="5"/>
-    <col width="30" customWidth="1" style="54" min="6" max="6"/>
-    <col width="13" customWidth="1" style="54" min="7" max="7"/>
-    <col width="30" customWidth="1" style="54" min="8" max="8"/>
-    <col width="13" customWidth="1" style="54" min="9" max="9"/>
-    <col width="30" customWidth="1" style="54" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1" s="54">
-      <c r="A1" s="56" t="inlineStr">
-        <is>
-          <t>Test cases — Parent — elementary (2–5 child)</t>
-        </is>
-      </c>
-      <c r="B1" s="57" t="n"/>
-      <c r="C1" s="57" t="n"/>
-      <c r="D1" s="57" t="n"/>
-      <c r="E1" s="57" t="n"/>
-      <c r="F1" s="57" t="n"/>
-      <c r="G1" s="57" t="n"/>
-      <c r="H1" s="57" t="n"/>
-      <c r="I1" s="57" t="n"/>
-      <c r="J1" s="57" t="n"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="54">
-      <c r="E2" s="58" t="inlineStr">
-        <is>
-          <t>Noreen Sultana
-Platform: ?</t>
-        </is>
-      </c>
-      <c r="F2" s="59" t="n"/>
-      <c r="G2" s="58" t="inlineStr">
-        <is>
-          <t>Tester 2
-Platform: ?</t>
-        </is>
-      </c>
-      <c r="H2" s="59" t="n"/>
-      <c r="I2" s="58" t="inlineStr">
-        <is>
-          <t>Tester 3
-Platform: ?</t>
-        </is>
-      </c>
-      <c r="J2" s="59" t="n"/>
-    </row>
-    <row r="3" ht="28" customHeight="1" s="54">
-      <c r="A3" s="60" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B3" s="60" t="inlineStr">
-        <is>
-          <t>User story</t>
-        </is>
-      </c>
-      <c r="C3" s="60" t="inlineStr">
-        <is>
-          <t>Steps to perform</t>
-        </is>
-      </c>
-      <c r="D3" s="60" t="inlineStr">
-        <is>
-          <t>Expected behavior (what you should see)</t>
-        </is>
-      </c>
-      <c r="E3" s="60" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="F3" s="60" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-      <c r="G3" s="60" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="H3" s="60" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-      <c r="I3" s="60" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="J3" s="60" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" s="54">
-      <c r="A4" s="61" t="inlineStr">
-        <is>
-          <t>Account &amp; access (all roles)</t>
-        </is>
-      </c>
-      <c r="B4" s="59" t="n"/>
-      <c r="C4" s="59" t="n"/>
-      <c r="D4" s="59" t="n"/>
-      <c r="E4" s="59" t="n"/>
-      <c r="F4" s="59" t="n"/>
-      <c r="G4" s="59" t="n"/>
-      <c r="H4" s="59" t="n"/>
-      <c r="I4" s="59" t="n"/>
-      <c r="J4" s="59" t="n"/>
-    </row>
-    <row r="5" ht="42" customHeight="1" s="54">
-      <c r="A5" s="62" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B5" s="63" t="inlineStr">
-        <is>
-          <t>As any user, I want to log in with email and password.</t>
-        </is>
-      </c>
-      <c r="C5" s="63" t="inlineStr">
-        <is>
-          <t>Enter valid email/password and Sign in.</t>
-        </is>
-      </c>
-      <c r="D5" s="63" t="inlineStr">
-        <is>
-          <t>You're signed in and taken to your role's home.</t>
-        </is>
-      </c>
-      <c r="E5" s="64" t="n"/>
-      <c r="F5" s="64" t="n"/>
-      <c r="G5" s="64" t="n"/>
-      <c r="H5" s="64" t="n"/>
-      <c r="I5" s="64" t="n"/>
-      <c r="J5" s="64" t="n"/>
-    </row>
-    <row r="6" ht="42" customHeight="1" s="54">
-      <c r="A6" s="62" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B6" s="63" t="inlineStr">
-        <is>
-          <t>As any user, I want to reveal my password while typing.</t>
-        </is>
-      </c>
-      <c r="C6" s="63" t="inlineStr">
-        <is>
-          <t>Tap the eye icon in the password field.</t>
-        </is>
-      </c>
-      <c r="D6" s="63" t="inlineStr">
-        <is>
-          <t>Password text toggles visible/hidden.</t>
-        </is>
-      </c>
-      <c r="E6" s="64" t="n"/>
-      <c r="F6" s="64" t="n"/>
-      <c r="G6" s="64" t="n"/>
-      <c r="H6" s="64" t="n"/>
-      <c r="I6" s="64" t="n"/>
-      <c r="J6" s="64" t="n"/>
-    </row>
-    <row r="7" ht="42" customHeight="1" s="54">
-      <c r="A7" s="62" t="inlineStr">
-        <is>
-          <t>AC3</t>
-        </is>
-      </c>
-      <c r="B7" s="63" t="inlineStr">
-        <is>
-          <t>As any user, I want to reset a forgotten password by email.</t>
-        </is>
-      </c>
-      <c r="C7" s="63" t="inlineStr">
-        <is>
-          <t>Forgot password → enter email → open email → follow link → set new password → sign in.</t>
-        </is>
-      </c>
-      <c r="D7" s="63" t="inlineStr">
-        <is>
-          <t>Reset email arrives; link works; new password signs in; old one fails.</t>
-        </is>
-      </c>
-      <c r="E7" s="64" t="n"/>
-      <c r="F7" s="64" t="n"/>
-      <c r="G7" s="64" t="n"/>
-      <c r="H7" s="64" t="n"/>
-      <c r="I7" s="64" t="n"/>
-      <c r="J7" s="64" t="n"/>
-    </row>
-    <row r="8" ht="42" customHeight="1" s="54">
-      <c r="A8" s="62" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B8" s="63" t="inlineStr">
-        <is>
-          <t>As any user, I want to sign out.</t>
-        </is>
-      </c>
-      <c r="C8" s="63" t="inlineStr">
-        <is>
-          <t>Use Sign out.</t>
-        </is>
-      </c>
-      <c r="D8" s="63" t="inlineStr">
-        <is>
-          <t>Logged out; returned to login/landing.</t>
-        </is>
-      </c>
-      <c r="E8" s="64" t="n"/>
-      <c r="F8" s="64" t="n"/>
-      <c r="G8" s="64" t="n"/>
-      <c r="H8" s="64" t="n"/>
-      <c r="I8" s="64" t="n"/>
-      <c r="J8" s="64" t="n"/>
-    </row>
-    <row r="9" ht="42" customHeight="1" s="54">
-      <c r="A9" s="62" t="inlineStr">
-        <is>
-          <t>AC5</t>
-        </is>
-      </c>
-      <c r="B9" s="63" t="inlineStr">
-        <is>
-          <t>As any user, I want a clear error for bad credentials.</t>
-        </is>
-      </c>
-      <c r="C9" s="63" t="inlineStr">
-        <is>
-          <t>Enter a wrong password.</t>
-        </is>
-      </c>
-      <c r="D9" s="63" t="inlineStr">
-        <is>
-          <t>Clear 'login failed' message; stay on login.</t>
-        </is>
-      </c>
-      <c r="E9" s="64" t="n"/>
-      <c r="F9" s="64" t="n"/>
-      <c r="G9" s="64" t="n"/>
-      <c r="H9" s="64" t="n"/>
-      <c r="I9" s="64" t="n"/>
-      <c r="J9" s="64" t="n"/>
-    </row>
-    <row r="10" ht="42" customHeight="1" s="54">
-      <c r="A10" s="62" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="B10" s="63" t="inlineStr">
-        <is>
-          <t>As any user, my session persists and protected pages are guarded.</t>
-        </is>
-      </c>
-      <c r="C10" s="63" t="inlineStr">
-        <is>
-          <t>Sign in, refresh; then sign out and open a protected URL directly.</t>
-        </is>
-      </c>
-      <c r="D10" s="63" t="inlineStr">
-        <is>
-          <t>Refresh stays signed in; protected pages redirect to login when signed out.</t>
-        </is>
-      </c>
-      <c r="E10" s="64" t="n"/>
-      <c r="F10" s="64" t="n"/>
-      <c r="G10" s="64" t="n"/>
-      <c r="H10" s="64" t="n"/>
-      <c r="I10" s="64" t="n"/>
-      <c r="J10" s="64" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" s="54">
-      <c r="A11" s="61" t="inlineStr">
-        <is>
-          <t>Parent — elementary (grades 2–5 child)</t>
-        </is>
-      </c>
-      <c r="B11" s="59" t="n"/>
-      <c r="C11" s="59" t="n"/>
-      <c r="D11" s="59" t="n"/>
-      <c r="E11" s="59" t="n"/>
-      <c r="F11" s="59" t="n"/>
-      <c r="G11" s="59" t="n"/>
-      <c r="H11" s="59" t="n"/>
-      <c r="I11" s="59" t="n"/>
-      <c r="J11" s="59" t="n"/>
-    </row>
-    <row r="12" ht="42" customHeight="1" s="54">
-      <c r="A12" s="62" t="inlineStr">
-        <is>
-          <t>PE1</t>
-        </is>
-      </c>
-      <c r="B12" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to register to manage my grade 2–5 child.</t>
-        </is>
-      </c>
-      <c r="C12" s="63" t="inlineStr">
-        <is>
-          <t>Create account → parent of a 2–5 child.</t>
-        </is>
-      </c>
-      <c r="D12" s="63" t="inlineStr">
-        <is>
-          <t>Parent account created.</t>
-        </is>
-      </c>
-      <c r="E12" s="64" t="n"/>
-      <c r="F12" s="64" t="n"/>
-      <c r="G12" s="64" t="n"/>
-      <c r="H12" s="64" t="n"/>
-      <c r="I12" s="64" t="n"/>
-      <c r="J12" s="64" t="n"/>
-    </row>
-    <row r="13" ht="42" customHeight="1" s="54">
-      <c r="A13" s="62" t="inlineStr">
-        <is>
-          <t>PE2</t>
-        </is>
-      </c>
-      <c r="B13" s="63" t="inlineStr">
-        <is>
-          <t>As an elementary parent, I want the right menu tabs.</t>
-        </is>
-      </c>
-      <c r="C13" s="63" t="inlineStr">
-        <is>
-          <t>Look at the left menu.</t>
-        </is>
-      </c>
-      <c r="D13" s="63" t="inlineStr">
-        <is>
-          <t>Dashboard and Find Opportunities (Help in footer).</t>
-        </is>
-      </c>
-      <c r="E13" s="64" t="n"/>
-      <c r="F13" s="64" t="n"/>
-      <c r="G13" s="64" t="n"/>
-      <c r="H13" s="64" t="n"/>
-      <c r="I13" s="64" t="n"/>
-      <c r="J13" s="64" t="n"/>
-    </row>
-    <row r="14" ht="42" customHeight="1" s="54">
-      <c r="A14" s="62" t="inlineStr">
-        <is>
-          <t>PE3</t>
-        </is>
-      </c>
-      <c r="B14" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to add a managed child (2–5).</t>
-        </is>
-      </c>
-      <c r="C14" s="63" t="inlineStr">
-        <is>
-          <t>Add child with name and grade (join code if required).</t>
-        </is>
-      </c>
-      <c r="D14" s="63" t="inlineStr">
-        <is>
-          <t>Child added; no separate login.</t>
-        </is>
-      </c>
-      <c r="E14" s="64" t="n"/>
-      <c r="F14" s="64" t="n"/>
-      <c r="G14" s="64" t="n"/>
-      <c r="H14" s="64" t="n"/>
-      <c r="I14" s="64" t="n"/>
-      <c r="J14" s="64" t="n"/>
-    </row>
-    <row r="15" ht="42" customHeight="1" s="54">
-      <c r="A15" s="62" t="inlineStr">
-        <is>
-          <t>PE4</t>
-        </is>
-      </c>
-      <c r="B15" s="63" t="inlineStr">
-        <is>
-          <t>As a parent with several kids, I want to switch child.</t>
-        </is>
-      </c>
-      <c r="C15" s="63" t="inlineStr">
-        <is>
-          <t>Use the child picker.</t>
-        </is>
-      </c>
-      <c r="D15" s="63" t="inlineStr">
-        <is>
-          <t>Selected child's context is used.</t>
-        </is>
-      </c>
-      <c r="E15" s="64" t="n"/>
-      <c r="F15" s="64" t="n"/>
-      <c r="G15" s="64" t="n"/>
-      <c r="H15" s="64" t="n"/>
-      <c r="I15" s="64" t="n"/>
-      <c r="J15" s="64" t="n"/>
-    </row>
-    <row r="16" ht="42" customHeight="1" s="54">
-      <c r="A16" s="62" t="inlineStr">
-        <is>
-          <t>PE5</t>
-        </is>
-      </c>
-      <c r="B16" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to sign my child up.</t>
-        </is>
-      </c>
-      <c r="C16" s="63" t="inlineStr">
-        <is>
-          <t>Find Opportunities → pick child → open event → sign up.</t>
-        </is>
-      </c>
-      <c r="D16" s="63" t="inlineStr">
-        <is>
-          <t>Child registered; appears on dashboard with calendar.</t>
-        </is>
-      </c>
-      <c r="E16" s="64" t="n"/>
-      <c r="F16" s="64" t="n"/>
-      <c r="G16" s="64" t="n"/>
-      <c r="H16" s="64" t="n"/>
-      <c r="I16" s="64" t="n"/>
-      <c r="J16" s="64" t="n"/>
-    </row>
-    <row r="17" ht="42" customHeight="1" s="54">
-      <c r="A17" s="62" t="inlineStr">
-        <is>
-          <t>PE6</t>
-        </is>
-      </c>
-      <c r="B17" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, child sign-up respects grade/org limits.</t>
-        </is>
-      </c>
-      <c r="C17" s="63" t="inlineStr">
-        <is>
-          <t>Try an ineligible event.</t>
-        </is>
-      </c>
-      <c r="D17" s="63" t="inlineStr">
-        <is>
-          <t>Hidden or blocked with a message.</t>
-        </is>
-      </c>
-      <c r="E17" s="64" t="n"/>
-      <c r="F17" s="64" t="n"/>
-      <c r="G17" s="64" t="n"/>
-      <c r="H17" s="64" t="n"/>
-      <c r="I17" s="64" t="n"/>
-      <c r="J17" s="64" t="n"/>
-    </row>
-    <row r="18" ht="42" customHeight="1" s="54">
-      <c r="A18" s="62" t="inlineStr">
-        <is>
-          <t>PE7</t>
-        </is>
-      </c>
-      <c r="B18" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to see my child's schedule.</t>
-        </is>
-      </c>
-      <c r="C18" s="63" t="inlineStr">
-        <is>
-          <t>Open the dashboard.</t>
-        </is>
-      </c>
-      <c r="D18" s="63" t="inlineStr">
-        <is>
-          <t>Child's upcoming events with add-to-calendar; new sign-ups flagged.</t>
-        </is>
-      </c>
-      <c r="E18" s="64" t="n"/>
-      <c r="F18" s="64" t="n"/>
-      <c r="G18" s="64" t="n"/>
-      <c r="H18" s="64" t="n"/>
-      <c r="I18" s="64" t="n"/>
-      <c r="J18" s="64" t="n"/>
-    </row>
-    <row r="19" ht="42" customHeight="1" s="54">
-      <c r="A19" s="62" t="inlineStr">
-        <is>
-          <t>PE8</t>
-        </is>
-      </c>
-      <c r="B19" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to invite a co-guardian.</t>
-        </is>
-      </c>
-      <c r="C19" s="63" t="inlineStr">
-        <is>
-          <t>Invite a co-guardian by email.</t>
-        </is>
-      </c>
-      <c r="D19" s="63" t="inlineStr">
-        <is>
-          <t>Invite email sent; on registering with that email they share access.</t>
-        </is>
-      </c>
-      <c r="E19" s="64" t="n"/>
-      <c r="F19" s="64" t="n"/>
-      <c r="G19" s="64" t="n"/>
-      <c r="H19" s="64" t="n"/>
-      <c r="I19" s="64" t="n"/>
-      <c r="J19" s="64" t="n"/>
-    </row>
-    <row r="20" ht="42" customHeight="1" s="54">
-      <c r="A20" s="62" t="inlineStr">
-        <is>
-          <t>PE9</t>
-        </is>
-      </c>
-      <c r="B20" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want notice when my child signs up.</t>
-        </is>
-      </c>
-      <c r="C20" s="63" t="inlineStr">
-        <is>
-          <t>Sign a child up (or have the other guardian do it).</t>
-        </is>
-      </c>
-      <c r="D20" s="63" t="inlineStr">
-        <is>
-          <t>A notification/confirmation is produced.</t>
-        </is>
-      </c>
-      <c r="E20" s="64" t="n"/>
-      <c r="F20" s="64" t="n"/>
-      <c r="G20" s="64" t="n"/>
-      <c r="H20" s="64" t="n"/>
-      <c r="I20" s="64" t="n"/>
-      <c r="J20" s="64" t="n"/>
-    </row>
-    <row r="21" ht="42" customHeight="1" s="54">
-      <c r="A21" s="62" t="inlineStr">
-        <is>
-          <t>PE10</t>
-        </is>
-      </c>
-      <c r="B21" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to submit my child's hours after an event (child has no login).</t>
-        </is>
-      </c>
-      <c r="C21" s="63" t="inlineStr">
-        <is>
-          <t>Dashboard → the child's 'Submit hours (past events)' → enter hours → Submit.</t>
-        </is>
-      </c>
-      <c r="D21" s="63" t="inlineStr">
-        <is>
-          <t>Hours go to the supervisor for approval; status shows 'Waiting for review'.</t>
-        </is>
-      </c>
-      <c r="E21" s="64" t="n"/>
-      <c r="F21" s="64" t="n"/>
-      <c r="G21" s="64" t="n"/>
-      <c r="H21" s="64" t="n"/>
-      <c r="I21" s="64" t="n"/>
-      <c r="J21" s="64" t="n"/>
-    </row>
-    <row r="22" ht="42" customHeight="1" s="54">
-      <c r="A22" s="62" t="inlineStr">
-        <is>
-          <t>PE11</t>
-        </is>
-      </c>
-      <c r="B22" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to resubmit my child's rejected hours.</t>
-        </is>
-      </c>
-      <c r="C22" s="63" t="inlineStr">
-        <is>
-          <t>On a rejected past event, enter corrected hours → Resubmit.</t>
-        </is>
-      </c>
-      <c r="D22" s="63" t="inlineStr">
-        <is>
-          <t>Returns to 'Waiting for review'.</t>
-        </is>
-      </c>
-      <c r="E22" s="64" t="n"/>
-      <c r="F22" s="64" t="n"/>
-      <c r="G22" s="64" t="n"/>
-      <c r="H22" s="64" t="n"/>
-      <c r="I22" s="64" t="n"/>
-      <c r="J22" s="64" t="n"/>
-    </row>
-    <row r="23" ht="42" customHeight="1" s="54">
-      <c r="A23" s="62" t="inlineStr">
-        <is>
-          <t>PE12</t>
-        </is>
-      </c>
-      <c r="B23" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to see each past event's hours status for my child.</t>
-        </is>
-      </c>
-      <c r="C23" s="63" t="inlineStr">
-        <is>
-          <t>Look at the child's past events list.</t>
-        </is>
-      </c>
-      <c r="D23" s="63" t="inlineStr">
-        <is>
-          <t>Each shows Approved / Waiting / Rejected as appropriate.</t>
-        </is>
-      </c>
-      <c r="E23" s="64" t="n"/>
-      <c r="F23" s="64" t="n"/>
-      <c r="G23" s="64" t="n"/>
-      <c r="H23" s="64" t="n"/>
-      <c r="I23" s="64" t="n"/>
-      <c r="J23" s="64" t="n"/>
-    </row>
-    <row r="24" ht="42" customHeight="1" s="54">
-      <c r="A24" s="62" t="inlineStr">
-        <is>
-          <t>PE13</t>
-        </is>
-      </c>
-      <c r="B24" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, all core participant actions are available to me for my child.</t>
-        </is>
-      </c>
-      <c r="C24" s="63" t="inlineStr">
-        <is>
-          <t>Confirm: browse, sign up, withdraw, add-to-calendar, submit hours, view progress toward medals.</t>
-        </is>
-      </c>
-      <c r="D24" s="63" t="inlineStr">
-        <is>
-          <t>All participant-style actions work on the child's behalf (the child never logs in).</t>
-        </is>
-      </c>
-      <c r="E24" s="64" t="n"/>
-      <c r="F24" s="64" t="n"/>
-      <c r="G24" s="64" t="n"/>
-      <c r="H24" s="64" t="n"/>
-      <c r="I24" s="64" t="n"/>
-      <c r="J24" s="64" t="n"/>
-    </row>
-    <row r="25" ht="42" customHeight="1" s="54">
-      <c r="A25" s="62" t="inlineStr">
-        <is>
-          <t>PE16</t>
-        </is>
-      </c>
-      <c r="B25" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to browse/search opportunities for my child (upcoming &amp; past).</t>
-        </is>
-      </c>
-      <c r="C25" s="63" t="inlineStr">
-        <is>
-          <t>Find Opportunities with the child selected; use search and the upcoming/past views.</t>
-        </is>
-      </c>
-      <c r="D25" s="63" t="inlineStr">
-        <is>
-          <t>Same event list a participant sees, scoped to the child's grade/org.</t>
-        </is>
-      </c>
-      <c r="E25" s="64" t="n"/>
-      <c r="F25" s="64" t="n"/>
-      <c r="G25" s="64" t="n"/>
-      <c r="H25" s="64" t="n"/>
-      <c r="I25" s="64" t="n"/>
-      <c r="J25" s="64" t="n"/>
-    </row>
-    <row r="26" ht="42" customHeight="1" s="54">
-      <c r="A26" s="62" t="inlineStr">
-        <is>
-          <t>PE17</t>
-        </is>
-      </c>
-      <c r="B26" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to withdraw my child from an event.</t>
-        </is>
-      </c>
-      <c r="C26" s="63" t="inlineStr">
-        <is>
-          <t>Open the child's upcoming events → withdraw.</t>
-        </is>
-      </c>
-      <c r="D26" s="63" t="inlineStr">
-        <is>
-          <t>The child is removed; the slot frees up.</t>
-        </is>
-      </c>
-      <c r="E26" s="64" t="n"/>
-      <c r="F26" s="64" t="n"/>
-      <c r="G26" s="64" t="n"/>
-      <c r="H26" s="64" t="n"/>
-      <c r="I26" s="64" t="n"/>
-      <c r="J26" s="64" t="n"/>
-    </row>
-    <row r="27" ht="42" customHeight="1" s="54">
-      <c r="A27" s="62" t="inlineStr">
-        <is>
-          <t>PE18</t>
-        </is>
-      </c>
-      <c r="B27" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to check my child in on event day.</t>
-        </is>
-      </c>
-      <c r="C27" s="63" t="inlineStr">
-        <is>
-          <t>On the event day within the window, check the child in.</t>
-        </is>
-      </c>
-      <c r="D27" s="63" t="inlineStr">
-        <is>
-          <t>Check-in succeeds for the child.</t>
-        </is>
-      </c>
-      <c r="E27" s="64" t="n"/>
-      <c r="F27" s="64" t="n"/>
-      <c r="G27" s="64" t="n"/>
-      <c r="H27" s="64" t="n"/>
-      <c r="I27" s="64" t="n"/>
-      <c r="J27" s="64" t="n"/>
-    </row>
-    <row r="28" ht="42" customHeight="1" s="54">
-      <c r="A28" s="62" t="inlineStr">
-        <is>
-          <t>PE19</t>
-        </is>
-      </c>
-      <c r="B28" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to see my child's medal progress.</t>
-        </is>
-      </c>
-      <c r="C28" s="63" t="inlineStr">
-        <is>
-          <t>Open the dashboard / child card.</t>
-        </is>
-      </c>
-      <c r="D28" s="63" t="inlineStr">
-        <is>
-          <t>Progress uses the child's grade-based thresholds (e.g. lower bar for younger grades).</t>
-        </is>
-      </c>
-      <c r="E28" s="64" t="n"/>
-      <c r="F28" s="64" t="n"/>
-      <c r="G28" s="64" t="n"/>
-      <c r="H28" s="64" t="n"/>
-      <c r="I28" s="64" t="n"/>
-      <c r="J28" s="64" t="n"/>
-    </row>
-    <row r="29" ht="42" customHeight="1" s="54">
-      <c r="A29" s="62" t="inlineStr">
-        <is>
-          <t>PE20</t>
-        </is>
-      </c>
-      <c r="B29" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, external &gt;5h for my child requires proof.</t>
-        </is>
-      </c>
-      <c r="C29" s="63" t="inlineStr">
-        <is>
-          <t>Outside hours for the child, over 5 hours, without then with a proof file.</t>
-        </is>
-      </c>
-      <c r="D29" s="63" t="inlineStr">
-        <is>
-          <t>Blocked without proof; submits with a photo/letter.</t>
-        </is>
-      </c>
-      <c r="E29" s="64" t="n"/>
-      <c r="F29" s="64" t="n"/>
-      <c r="G29" s="64" t="n"/>
-      <c r="H29" s="64" t="n"/>
-      <c r="I29" s="64" t="n"/>
-      <c r="J29" s="64" t="n"/>
-    </row>
-    <row r="30" ht="42" customHeight="1" s="54">
-      <c r="A30" s="62" t="inlineStr">
-        <is>
-          <t>PE14</t>
-        </is>
-      </c>
-      <c r="B30" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to log my child's outside/nonprofit volunteering.</t>
-        </is>
-      </c>
-      <c r="C30" s="63" t="inlineStr">
-        <is>
-          <t>Child card → 'Outside hours' → fill activity, org, date, hours, supervisor → Submit.</t>
-        </is>
-      </c>
-      <c r="D30" s="63" t="inlineStr">
-        <is>
-          <t>External hours submitted for the child and sent for supervisor approval (proof required over 5h).</t>
-        </is>
-      </c>
-      <c r="E30" s="64" t="n"/>
-      <c r="F30" s="64" t="n"/>
-      <c r="G30" s="64" t="n"/>
-      <c r="H30" s="64" t="n"/>
-      <c r="I30" s="64" t="n"/>
-      <c r="J30" s="64" t="n"/>
-    </row>
-    <row r="31" ht="42" customHeight="1" s="54">
-      <c r="A31" s="62" t="inlineStr">
-        <is>
-          <t>PE15</t>
-        </is>
-      </c>
-      <c r="B31" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want my child's verified service record.</t>
-        </is>
-      </c>
-      <c r="C31" s="63" t="inlineStr">
-        <is>
-          <t>Child card → 'Service record'.</t>
-        </is>
-      </c>
-      <c r="D31" s="63" t="inlineStr">
-        <is>
-          <t>The child's itemized record opens; Print / Save-as-PDF works.</t>
-        </is>
-      </c>
-      <c r="E31" s="64" t="n"/>
-      <c r="F31" s="64" t="n"/>
-      <c r="G31" s="64" t="n"/>
-      <c r="H31" s="64" t="n"/>
-      <c r="I31" s="64" t="n"/>
-      <c r="J31" s="64" t="n"/>
-    </row>
-    <row r="32" ht="42" customHeight="1" s="54">
-      <c r="A32" s="62" t="inlineStr">
-        <is>
-          <t>PE22</t>
-        </is>
-      </c>
-      <c r="B32" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to be emailed when my child's hours are reviewed.</t>
-        </is>
-      </c>
-      <c r="C32" s="63" t="inlineStr">
-        <is>
-          <t>Have a supervisor approve then reject a submission for a managed child.</t>
-        </is>
-      </c>
-      <c r="D32" s="63" t="inlineStr">
-        <is>
-          <t>You (the guardian) receive the approved / needs-attention emails, even though the child has no email of their own.</t>
-        </is>
-      </c>
-      <c r="E32" s="64" t="n"/>
-      <c r="F32" s="64" t="n"/>
-      <c r="G32" s="64" t="n"/>
-      <c r="H32" s="64" t="n"/>
-      <c r="I32" s="64" t="n"/>
-      <c r="J32" s="64" t="n"/>
-    </row>
-    <row r="33" ht="42" customHeight="1" s="54">
-      <c r="A33" s="62" t="inlineStr">
-        <is>
-          <t>PE23</t>
-        </is>
-      </c>
-      <c r="B33" s="63" t="inlineStr">
-        <is>
-          <t>As a parent, I want to edit my child's details.</t>
-        </is>
-      </c>
-      <c r="C33" s="63" t="inlineStr">
-        <is>
-          <t>Child card → Edit → change name/grade/school → save.</t>
-        </is>
-      </c>
-      <c r="D33" s="63" t="inlineStr">
-        <is>
-          <t>Changes save for the managed child.</t>
-        </is>
-      </c>
-      <c r="E33" s="64" t="n"/>
-      <c r="F33" s="64" t="n"/>
-      <c r="G33" s="64" t="n"/>
-      <c r="H33" s="64" t="n"/>
-      <c r="I33" s="64" t="n"/>
-      <c r="J33" s="64" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1" s="54">
-      <c r="A34" s="61" t="inlineStr">
-        <is>
-          <t>Cross-cutting</t>
-        </is>
-      </c>
-      <c r="B34" s="59" t="n"/>
-      <c r="C34" s="59" t="n"/>
-      <c r="D34" s="59" t="n"/>
-      <c r="E34" s="59" t="n"/>
-      <c r="F34" s="59" t="n"/>
-      <c r="G34" s="59" t="n"/>
-      <c r="H34" s="59" t="n"/>
-      <c r="I34" s="59" t="n"/>
-      <c r="J34" s="59" t="n"/>
-    </row>
-    <row r="35" ht="42" customHeight="1" s="54">
-      <c r="A35" s="62" t="inlineStr">
-        <is>
-          <t>X1</t>
-        </is>
-      </c>
-      <c r="B35" s="63" t="inlineStr">
-        <is>
-          <t>As a phone user, I want a usable mobile layout.</t>
-        </is>
-      </c>
-      <c r="C35" s="63" t="inlineStr">
-        <is>
-          <t>Open at phone width; use the menu drawer.</t>
-        </is>
-      </c>
-      <c r="D35" s="63" t="inlineStr">
-        <is>
-          <t>Layout adapts; drawer opens/closes; no horizontal scroll.</t>
-        </is>
-      </c>
-      <c r="E35" s="64" t="n"/>
-      <c r="F35" s="64" t="n"/>
-      <c r="G35" s="64" t="n"/>
-      <c r="H35" s="64" t="n"/>
-      <c r="I35" s="64" t="n"/>
-      <c r="J35" s="64" t="n"/>
-    </row>
-    <row r="36" ht="42" customHeight="1" s="54">
-      <c r="A36" s="62" t="inlineStr">
-        <is>
-          <t>X2</t>
-        </is>
-      </c>
-      <c r="B36" s="63" t="inlineStr">
-        <is>
-          <t>As a visitor, I want the recycling ribbon on the login page.</t>
-        </is>
-      </c>
-      <c r="C36" s="63" t="inlineStr">
-        <is>
-          <t>Open login signed out.</t>
-        </is>
-      </c>
-      <c r="D36" s="63" t="inlineStr">
-        <is>
-          <t>Green ribbon shows on login.</t>
-        </is>
-      </c>
-      <c r="E36" s="64" t="n"/>
-      <c r="F36" s="64" t="n"/>
-      <c r="G36" s="64" t="n"/>
-      <c r="H36" s="64" t="n"/>
-      <c r="I36" s="64" t="n"/>
-      <c r="J36" s="64" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A11:J11"/>
-  </mergeCells>
-  <conditionalFormatting sqref="E4:E36">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
-      <formula>"Pass"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
-      <formula>"Blocked"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:G36">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
-      <formula>"Pass"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
-      <formula>"Blocked"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I36">
+  <conditionalFormatting sqref="I4:I38">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4248,7 +4330,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E36 G4:G36 I4:I36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E38 G4:G38 I4:I38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6678,7 +6760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="54" min="1" max="1"/>
@@ -6965,7 +7047,7 @@
       </c>
       <c r="D12" s="63" t="inlineStr">
         <is>
-          <t>Dashboard, Reports, Users, Events, Organizations (Help in footer).</t>
+          <t>Dashboard, Reports, Users, Events, Organizations, Award Thresholds, Audit Log (Help in footer).</t>
         </is>
       </c>
       <c r="E12" s="64" t="n"/>
@@ -7007,17 +7089,17 @@
       </c>
       <c r="B14" s="63" t="inlineStr">
         <is>
-          <t>As a Super Admin, I want to create users incl. Supervisor and Super Admin.</t>
+          <t>As a Super Admin, I want to create users of any role.</t>
         </is>
       </c>
       <c r="C14" s="63" t="inlineStr">
         <is>
-          <t>Users → Add user → each role.</t>
+          <t>Users → Add user → open the Role list.</t>
         </is>
       </c>
       <c r="D14" s="63" t="inlineStr">
         <is>
-          <t>Participant/Supervisor/Super Admin options available; account created + invite email.</t>
+          <t>Participant, Supervisor, Admin, and Super Admin options are all available; account created + invite email.</t>
         </is>
       </c>
       <c r="E14" s="64" t="n"/>
@@ -7371,17 +7453,17 @@
       </c>
       <c r="B28" s="63" t="inlineStr">
         <is>
-          <t>As a Super Admin, creating a user pre-fills a temp password and emails an invite.</t>
+          <t>As a Super Admin, creating a user auto-fills a temp password per role and emails an invite.</t>
         </is>
       </c>
       <c r="C28" s="63" t="inlineStr">
         <is>
-          <t>Add user; note the temp password field is pre-filled (Supervisor123!); save.</t>
+          <t>Add user; change the Role and watch the temp password auto-fill (Supervisor→Supervisor123!, Participant→Participant123!, Admin→Admin123!, Super Admin→SuperAdmin123!); save.</t>
         </is>
       </c>
       <c r="D28" s="63" t="inlineStr">
         <is>
-          <t>Account created; the person gets a set-password invite email.</t>
+          <t>Password auto-fills to match the role (and is editable); the browser does NOT autofill your own email/password; account created; the person gets a set-password invite email.</t>
         </is>
       </c>
       <c r="E28" s="64" t="n"/>
@@ -7407,7 +7489,7 @@
       </c>
       <c r="D29" s="63" t="inlineStr">
         <is>
-          <t>The user is stamped to that org (visible/manageable by that org's Admin).</t>
+          <t>The Organization field is shown; the user is stamped to that org. Creating an 'Admin' with an org makes them manage that org.</t>
         </is>
       </c>
       <c r="E29" s="64" t="n"/>
@@ -7415,65 +7497,65 @@
       <c r="G29" s="64" t="n"/>
       <c r="H29" s="64" t="n"/>
     </row>
-    <row r="30" ht="20" customHeight="1" s="54">
-      <c r="A30" s="61" t="inlineStr">
+    <row r="30" ht="42" customHeight="1" s="54">
+      <c r="A30" s="62" t="inlineStr">
+        <is>
+          <t>SA19</t>
+        </is>
+      </c>
+      <c r="B30" s="63" t="inlineStr">
+        <is>
+          <t>As a Super Admin, I want to add a specific participant to an event by email.</t>
+        </is>
+      </c>
+      <c r="C30" s="63" t="inlineStr">
+        <is>
+          <t>Open an event's Roster → Add a participant → enter a participant's account email → Add.</t>
+        </is>
+      </c>
+      <c r="D30" s="63" t="inlineStr">
+        <is>
+          <t>They're registered and emailed ('added to &lt;event&gt;'); it appears in their schedule. A managed elementary child (no email) can't be added this way — a guardian signs them up instead.</t>
+        </is>
+      </c>
+      <c r="E30" s="64" t="n"/>
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="64" t="n"/>
+      <c r="H30" s="64" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" s="54">
+      <c r="A31" s="61" t="inlineStr">
         <is>
           <t>Cross-cutting</t>
         </is>
       </c>
-      <c r="B30" s="59" t="n"/>
-      <c r="C30" s="59" t="n"/>
-      <c r="D30" s="59" t="n"/>
-      <c r="E30" s="59" t="n"/>
-      <c r="F30" s="59" t="n"/>
-      <c r="G30" s="59" t="n"/>
-      <c r="H30" s="59" t="n"/>
-    </row>
-    <row r="31" ht="42" customHeight="1" s="54">
-      <c r="A31" s="62" t="inlineStr">
-        <is>
-          <t>X1</t>
-        </is>
-      </c>
-      <c r="B31" s="63" t="inlineStr">
-        <is>
-          <t>As a phone user, I want a usable mobile layout.</t>
-        </is>
-      </c>
-      <c r="C31" s="63" t="inlineStr">
-        <is>
-          <t>Open at phone width; use the menu drawer.</t>
-        </is>
-      </c>
-      <c r="D31" s="63" t="inlineStr">
-        <is>
-          <t>Layout adapts; drawer opens/closes; no horizontal scroll.</t>
-        </is>
-      </c>
-      <c r="E31" s="64" t="n"/>
-      <c r="F31" s="64" t="n"/>
-      <c r="G31" s="64" t="n"/>
-      <c r="H31" s="64" t="n"/>
+      <c r="B31" s="59" t="n"/>
+      <c r="C31" s="59" t="n"/>
+      <c r="D31" s="59" t="n"/>
+      <c r="E31" s="59" t="n"/>
+      <c r="F31" s="59" t="n"/>
+      <c r="G31" s="59" t="n"/>
+      <c r="H31" s="59" t="n"/>
     </row>
     <row r="32" ht="42" customHeight="1" s="54">
       <c r="A32" s="62" t="inlineStr">
         <is>
-          <t>X2</t>
+          <t>X1</t>
         </is>
       </c>
       <c r="B32" s="63" t="inlineStr">
         <is>
-          <t>As a visitor, I want the recycling ribbon on the login page.</t>
+          <t>As a phone user, I want a usable mobile layout.</t>
         </is>
       </c>
       <c r="C32" s="63" t="inlineStr">
         <is>
-          <t>Open login signed out.</t>
+          <t>Open at phone width; use the menu drawer.</t>
         </is>
       </c>
       <c r="D32" s="63" t="inlineStr">
         <is>
-          <t>Green ribbon shows on login.</t>
+          <t>Layout adapts; drawer opens/closes; no horizontal scroll.</t>
         </is>
       </c>
       <c r="E32" s="64" t="n"/>
@@ -7481,16 +7563,42 @@
       <c r="G32" s="64" t="n"/>
       <c r="H32" s="64" t="n"/>
     </row>
+    <row r="33" ht="42" customHeight="1" s="54">
+      <c r="A33" s="62" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="B33" s="63" t="inlineStr">
+        <is>
+          <t>As a visitor, I want the recycling ribbon on the login page.</t>
+        </is>
+      </c>
+      <c r="C33" s="63" t="inlineStr">
+        <is>
+          <t>Open login signed out.</t>
+        </is>
+      </c>
+      <c r="D33" s="63" t="inlineStr">
+        <is>
+          <t>Green ribbon shows on login.</t>
+        </is>
+      </c>
+      <c r="E33" s="64" t="n"/>
+      <c r="F33" s="64" t="n"/>
+      <c r="G33" s="64" t="n"/>
+      <c r="H33" s="64" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A30:H30"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A31:H31"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E32">
+  <conditionalFormatting sqref="E4:E33">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Pass"</formula>
     </cfRule>
@@ -7501,7 +7609,7 @@
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4:G32">
+  <conditionalFormatting sqref="G4:G33">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Pass"</formula>
     </cfRule>
@@ -7513,7 +7621,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E32 G4:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E33 G4:G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7610,7 +7718,7 @@
         </is>
       </c>
       <c r="B5" s="69" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="69" t="n">
         <v>2</v>
@@ -7643,7 +7751,7 @@
         </is>
       </c>
       <c r="B6" s="69" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" s="69" t="n">
         <v>3</v>
@@ -7775,7 +7883,7 @@
         </is>
       </c>
       <c r="B10" s="69" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="69" t="n">
         <v>2</v>

</xml_diff>